<commit_message>
Norway nitrogen mirror exports and one EUR/USD rate for the lost-fuel anchors
- nitrogen_consumption: Norway's exports from partner mirror flows (own report
  3 kt N vs 0.63 Mt N reported by 112 partners); Norway becomes a net exporter
  of the ammonia chain. ammonia_consumption: Central African Rep. name fix.
  patch_nitrogen_2026_10_19 applies both to data/cost.
- security: ACER and ENTSOG anchors at the 2025 average 1.13 US$/EUR used for
  carbon prices (ENTSOG 175 -> 188.3 US$/GJ, ACER 22.0 -> 21.7 US$/GJ).
- make_tab_breakeven: anchors and the 2022 peak (2025 US$) from the code.
- Rebuilt all cases and SI analyses (work/rebuild_*_2026_10_19.sh); Source
  Data regenerated; test_paper expectations updated (9 justified at 2030,
  15 of 26 above US$100/t, 0.55/1.26/1.91 Gt).
- data/cost: corridors_discussion, ed_crisis_* and supply_demand synced with
  the published case outputs (case_low build had copied stale versions).
</commit_message>
<xml_diff>
--- a/source_data/Fig3.xlsx
+++ b/source_data/Fig3.xlsx
@@ -656,10 +656,10 @@
         <v>6.423</v>
       </c>
       <c r="S2" t="n">
-        <v>30.414</v>
+        <v>30.54</v>
       </c>
       <c r="T2" t="n">
-        <v>1.56</v>
+        <v>1.566</v>
       </c>
       <c r="U2" t="inlineStr">
         <is>
@@ -725,10 +725,10 @@
         <v>17.6</v>
       </c>
       <c r="S3" t="n">
-        <v>14.547</v>
+        <v>14.607</v>
       </c>
       <c r="T3" t="n">
-        <v>0.473</v>
+        <v>0.475</v>
       </c>
       <c r="U3" t="inlineStr">
         <is>
@@ -794,10 +794,10 @@
         <v>71.18300000000001</v>
       </c>
       <c r="S4" t="n">
-        <v>17.855</v>
+        <v>17.929</v>
       </c>
       <c r="T4" t="n">
-        <v>4.513</v>
+        <v>4.532</v>
       </c>
       <c r="U4" t="inlineStr">
         <is>
@@ -863,10 +863,10 @@
         <v>97.60899999999999</v>
       </c>
       <c r="S5" t="n">
-        <v>0.754</v>
+        <v>0.757</v>
       </c>
       <c r="T5" t="n">
-        <v>0.17</v>
+        <v>0.171</v>
       </c>
       <c r="U5" t="inlineStr">
         <is>
@@ -932,10 +932,10 @@
         <v>96.11</v>
       </c>
       <c r="S6" t="n">
-        <v>1.732</v>
+        <v>1.739</v>
       </c>
       <c r="T6" t="n">
-        <v>0.343</v>
+        <v>0.344</v>
       </c>
       <c r="U6" t="inlineStr">
         <is>
@@ -1001,10 +1001,10 @@
         <v>100</v>
       </c>
       <c r="S7" t="n">
-        <v>0.639</v>
+        <v>0.642</v>
       </c>
       <c r="T7" t="n">
-        <v>0.342</v>
+        <v>0.343</v>
       </c>
       <c r="U7" t="inlineStr">
         <is>
@@ -1070,10 +1070,10 @@
         <v>95.849</v>
       </c>
       <c r="S8" t="n">
-        <v>5.912</v>
+        <v>5.936</v>
       </c>
       <c r="T8" t="n">
-        <v>2.593</v>
+        <v>2.604</v>
       </c>
       <c r="U8" t="inlineStr">
         <is>
@@ -1139,10 +1139,10 @@
         <v>0</v>
       </c>
       <c r="S9" t="n">
-        <v>1.955</v>
+        <v>1.963</v>
       </c>
       <c r="T9" t="n">
-        <v>1.352</v>
+        <v>1.358</v>
       </c>
       <c r="U9" t="inlineStr">
         <is>
@@ -1208,10 +1208,10 @@
         <v>97.947</v>
       </c>
       <c r="S10" t="n">
-        <v>0.491</v>
+        <v>0.493</v>
       </c>
       <c r="T10" t="n">
-        <v>0.192</v>
+        <v>0.193</v>
       </c>
       <c r="U10" t="inlineStr">
         <is>
@@ -1277,10 +1277,10 @@
         <v>99.905</v>
       </c>
       <c r="S11" t="n">
-        <v>0.554</v>
+        <v>0.5570000000000001</v>
       </c>
       <c r="T11" t="n">
-        <v>0.291</v>
+        <v>0.292</v>
       </c>
       <c r="U11" t="inlineStr">
         <is>
@@ -1349,7 +1349,7 @@
         <v>0.068</v>
       </c>
       <c r="T12" t="n">
-        <v>0.111</v>
+        <v>0.112</v>
       </c>
       <c r="U12" t="inlineStr">
         <is>
@@ -1415,10 +1415,10 @@
         <v>69.146</v>
       </c>
       <c r="S13" t="n">
-        <v>0.35</v>
+        <v>0.352</v>
       </c>
       <c r="T13" t="n">
-        <v>0.263</v>
+        <v>0.264</v>
       </c>
       <c r="U13" t="inlineStr">
         <is>
@@ -1484,10 +1484,10 @@
         <v>84.604</v>
       </c>
       <c r="S14" t="n">
-        <v>1.318</v>
+        <v>1.324</v>
       </c>
       <c r="T14" t="n">
-        <v>1.273</v>
+        <v>1.278</v>
       </c>
       <c r="U14" t="inlineStr">
         <is>
@@ -1553,10 +1553,10 @@
         <v>97.666</v>
       </c>
       <c r="S15" t="n">
-        <v>0.577</v>
+        <v>0.579</v>
       </c>
       <c r="T15" t="n">
-        <v>0.144</v>
+        <v>0.145</v>
       </c>
       <c r="U15" t="inlineStr">
         <is>
@@ -1622,10 +1622,10 @@
         <v>15.4</v>
       </c>
       <c r="S16" t="n">
-        <v>1.153</v>
+        <v>1.157</v>
       </c>
       <c r="T16" t="n">
-        <v>2.24</v>
+        <v>2.249</v>
       </c>
       <c r="U16" t="inlineStr">
         <is>
@@ -1691,10 +1691,10 @@
         <v>20.514</v>
       </c>
       <c r="S17" t="n">
-        <v>0.967</v>
+        <v>0.971</v>
       </c>
       <c r="T17" t="n">
-        <v>2.646</v>
+        <v>2.657</v>
       </c>
       <c r="U17" t="inlineStr">
         <is>
@@ -1760,10 +1760,10 @@
         <v>32.194</v>
       </c>
       <c r="S18" t="n">
-        <v>2.748</v>
+        <v>2.759</v>
       </c>
       <c r="T18" t="n">
-        <v>6.747</v>
+        <v>6.775</v>
       </c>
       <c r="U18" t="inlineStr">
         <is>
@@ -1829,10 +1829,10 @@
         <v>100</v>
       </c>
       <c r="S19" t="n">
-        <v>0.12</v>
+        <v>0.121</v>
       </c>
       <c r="T19" t="n">
-        <v>0.885</v>
+        <v>0.889</v>
       </c>
       <c r="U19" t="inlineStr">
         <is>
@@ -1898,10 +1898,10 @@
         <v>100</v>
       </c>
       <c r="S20" t="n">
-        <v>0.422</v>
+        <v>0.424</v>
       </c>
       <c r="T20" t="n">
-        <v>0.866</v>
+        <v>0.87</v>
       </c>
       <c r="U20" t="inlineStr">
         <is>
@@ -1970,7 +1970,7 @@
         <v>0.139</v>
       </c>
       <c r="T21" t="n">
-        <v>1.275</v>
+        <v>1.281</v>
       </c>
       <c r="U21" t="inlineStr">
         <is>
@@ -2039,7 +2039,7 @@
         <v>0.021</v>
       </c>
       <c r="T22" t="n">
-        <v>0.167</v>
+        <v>0.168</v>
       </c>
       <c r="U22" t="inlineStr">
         <is>
@@ -2108,7 +2108,7 @@
         <v>0.011</v>
       </c>
       <c r="T23" t="n">
-        <v>0.569</v>
+        <v>0.571</v>
       </c>
       <c r="U23" t="inlineStr">
         <is>
@@ -2174,10 +2174,10 @@
         <v>100</v>
       </c>
       <c r="S24" t="n">
-        <v>0.18</v>
+        <v>0.181</v>
       </c>
       <c r="T24" t="n">
-        <v>0.249</v>
+        <v>0.25</v>
       </c>
       <c r="U24" t="inlineStr">
         <is>
@@ -2243,10 +2243,10 @@
         <v>100</v>
       </c>
       <c r="S25" t="n">
-        <v>0.418</v>
+        <v>0.419</v>
       </c>
       <c r="T25" t="n">
-        <v>1.168</v>
+        <v>1.173</v>
       </c>
       <c r="U25" t="inlineStr">
         <is>
@@ -2312,10 +2312,10 @@
         <v>100</v>
       </c>
       <c r="S26" t="n">
-        <v>0.126</v>
+        <v>0.127</v>
       </c>
       <c r="T26" t="n">
-        <v>0.6919999999999999</v>
+        <v>0.694</v>
       </c>
       <c r="U26" t="inlineStr">
         <is>
@@ -2381,10 +2381,10 @@
         <v>55</v>
       </c>
       <c r="S27" t="n">
-        <v>2.322</v>
+        <v>2.332</v>
       </c>
       <c r="T27" t="n">
-        <v>1.291</v>
+        <v>1.297</v>
       </c>
       <c r="U27" t="inlineStr">
         <is>
@@ -2450,10 +2450,10 @@
         <v>0</v>
       </c>
       <c r="S28" t="n">
-        <v>0.17</v>
+        <v>0.171</v>
       </c>
       <c r="T28" t="n">
-        <v>0.133</v>
+        <v>0.134</v>
       </c>
       <c r="U28" t="inlineStr">
         <is>
@@ -2519,10 +2519,10 @@
         <v>75.36</v>
       </c>
       <c r="S29" t="n">
-        <v>0.631</v>
+        <v>0.634</v>
       </c>
       <c r="T29" t="n">
-        <v>1.478</v>
+        <v>1.484</v>
       </c>
       <c r="U29" t="inlineStr">
         <is>
@@ -2582,16 +2582,16 @@
         <v>99.82599999999999</v>
       </c>
       <c r="Q30" t="n">
-        <v>0.382</v>
+        <v>0</v>
       </c>
       <c r="R30" t="n">
-        <v>61.9</v>
+        <v>0</v>
       </c>
       <c r="S30" t="n">
-        <v>0.592</v>
+        <v>0.151</v>
       </c>
       <c r="T30" t="n">
-        <v>1.115</v>
+        <v>0.285</v>
       </c>
       <c r="U30" t="inlineStr">
         <is>
@@ -2660,7 +2660,7 @@
         <v>0.022</v>
       </c>
       <c r="T31" t="n">
-        <v>0.202</v>
+        <v>0.203</v>
       </c>
       <c r="U31" t="inlineStr">
         <is>

</xml_diff>